<commit_message>
Reorganizing files to create CEA and SLE screening with the predictive capabilities of the MTGPR.
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91857889-0EA8-4489-B573-EC8153478EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FDFD30-85F6-41FB-BCFA-43AB1E01FA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="Unfinished CATALOG" sheetId="1" r:id="rId1"/>
@@ -883,387 +883,8 @@
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Alexander Glotov</author>
-  </authors>
-  <commentList>
-    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{5501DECC-CA51-4608-A2A9-124DF8574F9C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Ashlee</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{366F9C8A-C349-48E6-8883-C6E40BE5B81F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Ashlee</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{F3DAE571-D049-4F99-B2BB-AD33D024F8CA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=1912</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{FC2E5BC0-6FB5-46E6-A96C-B5A571D6D42E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{97513E38-6E68-43E5-A94C-6F8C909B7BCE}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{1DBE5D3C-786F-4099-B286-532040D0D3AF}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{E40BDC6B-934E-411C-B492-C5CD43E5E926}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Hilgeman, Mouroux, Mok, Holan</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E4" authorId="0" shapeId="0" xr:uid="{9BE4DF8B-2AFF-4A6C-9B30-43F0C8BC4258}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Hilgeman, Mouroux, Mok, Holan</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{22C3A041-08B4-4358-8FFC-0CCF2BF68560}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C288324&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{9B46E2A3-89E8-410D-9F36-E3CC4EDF12E7}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{7AFC09FE-6D63-4AB4-9F34-8C6E6346C5F6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://www.sciencedirect.com/science/article/pii/S1750583613004258</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{19F57934-8119-42AF-9A95-961B9A767839}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C141435&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{A44F0865-2292-4150-8EDA-994F95E330D4}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Ashlee</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{22EA6CA3-1836-4119-B6E7-99ADB8AE94F6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Ashlee</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{7A8F76C3-1C0D-4DE3-9D30-F2E27379947A}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://atct.anl.gov/Thermochemical%20Data/version%201.220/species/?species_number=1907</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="90">
   <si>
     <t>Full Name</t>
   </si>
@@ -1497,6 +1118,45 @@
   </si>
   <si>
     <t>[BH4-].[K+]</t>
+  </si>
+  <si>
+    <t>Melting Temperature STDEV [K]</t>
+  </si>
+  <si>
+    <t>Melting Temperature Count</t>
+  </si>
+  <si>
+    <t>Enthalpy of Fusion [kJ/mol]</t>
+  </si>
+  <si>
+    <t>Enthalpy of Fusion STDEV [kJ/mol]</t>
+  </si>
+  <si>
+    <t>Enthalpy of Fusion Count</t>
+  </si>
+  <si>
+    <t>Enthalpy of Formation STDEV [kJ/mol]</t>
+  </si>
+  <si>
+    <t>Enthalpy of Formation Count</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium borohydride</t>
+  </si>
+  <si>
+    <t>Melting Temperature [K]</t>
+  </si>
+  <si>
+    <t>Enthalpy of Formation [kJ/mol]</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium chloride</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>ammonia borane</t>
   </si>
 </sst>
 </file>
@@ -2474,19 +2134,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE786A1-84C7-4241-A3B9-138356725320}">
-  <dimension ref="A1:F6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE786A1-84C7-4241-A3B9-138356725320}">
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="11" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2497,110 +2162,58 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>85</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2">
-        <f>79+273.15</f>
-        <v>352.15</v>
-      </c>
-      <c r="E2">
-        <v>7730</v>
-      </c>
-      <c r="F2">
-        <v>-315890</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3">
-        <v>284.2</v>
-      </c>
-      <c r="E3">
-        <v>21830</v>
-      </c>
-      <c r="F3">
-        <v>-63010</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4">
-        <v>363.7</v>
-      </c>
-      <c r="E4">
-        <v>12500</v>
-      </c>
-      <c r="F4">
-        <v>49800</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5">
-        <v>283.45999999999998</v>
-      </c>
-      <c r="E5">
-        <v>13800</v>
-      </c>
-      <c r="F5">
-        <v>-507500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <f>133+273.15</f>
-        <v>406.15</v>
-      </c>
-      <c r="E6">
-        <v>10340</v>
-      </c>
-      <c r="F6">
-        <v>-333330</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added the ability to use HANNA. HANNA lacks the ability to obtain close enough activity coefficients. Will require additional fine tuning. Also added phase diagram data to help with activity coefficient predictions.
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FDFD30-85F6-41FB-BCFA-43AB1E01FA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82934A1-3E9D-4F5D-96C2-17F125CE508B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="Unfinished CATALOG" sheetId="1" r:id="rId1"/>
-    <sheet name="Input" sheetId="2" r:id="rId2"/>
+    <sheet name="Pure Input" sheetId="2" r:id="rId2"/>
+    <sheet name="Binary Input" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unfinished CATALOG'!$A$1:$F$1</definedName>
@@ -56,7 +57,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -65,7 +66,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://pubchem.ncbi.nlm.nih.gov/compound/Water#section=Melting-Point</t>
@@ -80,7 +81,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -89,7 +90,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.engineeringtoolbox.com/water-thermal-properties-d_162.html</t>
@@ -129,7 +130,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -138,7 +139,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Ashlee</t>
@@ -153,7 +154,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -162,7 +163,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Ashlee</t>
@@ -202,7 +203,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -211,7 +212,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Ashlee</t>
@@ -226,7 +227,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -235,7 +236,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Ashlee</t>
@@ -275,7 +276,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -284,7 +285,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Hilgeman, Mouroux, Mok, Holan</t>
@@ -299,7 +300,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -308,7 +309,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Hilgeman, Mouroux, Mok, Holan</t>
@@ -423,7 +424,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -432,7 +433,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
@@ -447,7 +448,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -456,7 +457,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
@@ -471,7 +472,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -480,7 +481,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
@@ -570,7 +571,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -579,7 +580,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
@@ -594,7 +595,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -603,7 +604,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
@@ -618,7 +619,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -627,7 +628,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=2#Thermo-Condensed</t>
@@ -642,7 +643,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -651,7 +652,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C112492&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
@@ -666,7 +667,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -675,7 +676,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C112492&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
@@ -766,7 +767,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -775,7 +776,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 1)https://iris.unito.it/bitstream/2318/1995351/2/Dematteis%20-%20PhD%20Thesis%20-%20DEF_REFEREE.pdf</t>
@@ -790,7 +791,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -799,7 +800,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 1)https://iris.unito.it/bitstream/2318/1995351/2/Dematteis%20-%20PhD%20Thesis%20-%20DEF_REFEREE.pdf</t>
@@ -839,7 +840,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -848,7 +849,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C1643192&amp;Mask=1EFF#Thermo-Gas</t>
@@ -863,7 +864,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Alexander Glotov:</t>
         </r>
@@ -872,7 +873,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://webbook.nist.gov/cgi/cbook.cgi?ID=C1643192&amp;Mask=1EFF#Thermo-Gas</t>
@@ -884,7 +885,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="109">
   <si>
     <t>Full Name</t>
   </si>
@@ -1141,9 +1142,6 @@
     <t>Enthalpy of Formation Count</t>
   </si>
   <si>
-    <t>tetrabutylammonium borohydride</t>
-  </si>
-  <si>
     <t>Melting Temperature [K]</t>
   </si>
   <si>
@@ -1156,14 +1154,74 @@
     <t>CCCC[N+](CCCC)(CCCC)CCCC.[Cl-]</t>
   </si>
   <si>
-    <t>ammonia borane</t>
+    <t>tetramethylammonium chloride</t>
+  </si>
+  <si>
+    <t>tetraethylammonium bromide</t>
+  </si>
+  <si>
+    <t>tetrapropylammonium bromide</t>
+  </si>
+  <si>
+    <t>tetraethylammonium chloride</t>
+  </si>
+  <si>
+    <t>tetrapropylammonium chloride</t>
+  </si>
+  <si>
+    <t>potassium chloride</t>
+  </si>
+  <si>
+    <t>lithium chloride</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[Cl-]</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[Br-]</t>
+  </si>
+  <si>
+    <t>CCC[N+](CCC)(CCC)CCC.[Br-]</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[Cl-]</t>
+  </si>
+  <si>
+    <t>CCC[N+](CCC)(CCC)CCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>[K+].[Cl-]</t>
+  </si>
+  <si>
+    <t>[Li+].[Cl-]</t>
+  </si>
+  <si>
+    <t>Chemical (1)</t>
+  </si>
+  <si>
+    <t>Chemical (2)</t>
+  </si>
+  <si>
+    <t>Composition (1)</t>
+  </si>
+  <si>
+    <t>Composition (2)</t>
+  </si>
+  <si>
+    <t>Temperature</t>
+  </si>
+  <si>
+    <t>Temperature Unit</t>
+  </si>
+  <si>
+    <t>K</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1189,19 +1247,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2135,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE786A1-84C7-4241-A3B9-138356725320}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.28515625" bestFit="1" customWidth="1"/>
@@ -2162,7 +2207,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>77</v>
@@ -2180,7 +2225,7 @@
         <v>81</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>82</v>
@@ -2191,18 +2236,18 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
         <v>87</v>
-      </c>
-      <c r="C3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -2210,7 +2255,1344 @@
         <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{664E3DE9-D4FA-47AC-BF11-BE862F2429E3}">
+  <dimension ref="A1:F64"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2">
+        <v>0.95</v>
+      </c>
+      <c r="D2">
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="E2">
+        <v>585.5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3">
+        <v>0.90400000000000003</v>
+      </c>
+      <c r="D3">
+        <v>9.5999999999999974E-2</v>
+      </c>
+      <c r="E3">
+        <v>520.70000000000005</v>
+      </c>
+      <c r="F3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4">
+        <v>0.85</v>
+      </c>
+      <c r="D4">
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="E4">
+        <v>482</v>
+      </c>
+      <c r="F4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5">
+        <v>0.78700000000000003</v>
+      </c>
+      <c r="D5">
+        <v>0.21299999999999997</v>
+      </c>
+      <c r="E5">
+        <v>436</v>
+      </c>
+      <c r="F5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6">
+        <v>0.72299999999999998</v>
+      </c>
+      <c r="D6">
+        <v>0.27700000000000002</v>
+      </c>
+      <c r="E6">
+        <v>398</v>
+      </c>
+      <c r="F6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7">
+        <v>0.63400000000000001</v>
+      </c>
+      <c r="D7">
+        <v>0.36599999999999999</v>
+      </c>
+      <c r="E7">
+        <v>362.8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8">
+        <v>0.52</v>
+      </c>
+      <c r="D8">
+        <v>0.48</v>
+      </c>
+      <c r="E8">
+        <v>344.8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="D9">
+        <v>0.59200000000000008</v>
+      </c>
+      <c r="E9">
+        <v>343.7</v>
+      </c>
+      <c r="F9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="D10">
+        <v>0.75800000000000001</v>
+      </c>
+      <c r="E10">
+        <v>342.4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="D11">
+        <v>5.1000000000000045E-2</v>
+      </c>
+      <c r="E11">
+        <v>609.70000000000005</v>
+      </c>
+      <c r="F11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12">
+        <v>0.89900000000000002</v>
+      </c>
+      <c r="D12">
+        <v>0.10099999999999998</v>
+      </c>
+      <c r="E12">
+        <v>608.79999999999995</v>
+      </c>
+      <c r="F12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13">
+        <v>0.8</v>
+      </c>
+      <c r="D13">
+        <v>0.19999999999999996</v>
+      </c>
+      <c r="E13">
+        <v>595.70000000000005</v>
+      </c>
+      <c r="F13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="D14">
+        <v>0.30100000000000005</v>
+      </c>
+      <c r="E14">
+        <v>574.4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15">
+        <v>0.6</v>
+      </c>
+      <c r="D15">
+        <v>0.4</v>
+      </c>
+      <c r="E15">
+        <v>547.9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16">
+        <v>0.501</v>
+      </c>
+      <c r="D16">
+        <v>0.499</v>
+      </c>
+      <c r="E16">
+        <v>517.79999999999995</v>
+      </c>
+      <c r="F16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="D17">
+        <v>0.59699999999999998</v>
+      </c>
+      <c r="E17">
+        <v>488</v>
+      </c>
+      <c r="F17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18">
+        <v>0.3</v>
+      </c>
+      <c r="D18">
+        <v>0.7</v>
+      </c>
+      <c r="E18">
+        <v>515.9</v>
+      </c>
+      <c r="F18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19">
+        <v>0.2</v>
+      </c>
+      <c r="D19">
+        <v>0.8</v>
+      </c>
+      <c r="E19">
+        <v>538.5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="D20">
+        <v>0.89900000000000002</v>
+      </c>
+      <c r="E20">
+        <v>554.20000000000005</v>
+      </c>
+      <c r="F20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="D21">
+        <v>5.1000000000000045E-2</v>
+      </c>
+      <c r="E21">
+        <v>600.9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22">
+        <v>0.9</v>
+      </c>
+      <c r="D22">
+        <v>9.9999999999999978E-2</v>
+      </c>
+      <c r="E22">
+        <v>595</v>
+      </c>
+      <c r="F22" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23">
+        <v>0.8</v>
+      </c>
+      <c r="D23">
+        <v>0.19999999999999996</v>
+      </c>
+      <c r="E23">
+        <v>579.6</v>
+      </c>
+      <c r="F23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24">
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="D24">
+        <v>0.30200000000000005</v>
+      </c>
+      <c r="E24">
+        <v>557.9</v>
+      </c>
+      <c r="F24" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25">
+        <v>0.59899999999999998</v>
+      </c>
+      <c r="D25">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="E25">
+        <v>531.1</v>
+      </c>
+      <c r="F25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26">
+        <v>0.501</v>
+      </c>
+      <c r="D26">
+        <v>0.499</v>
+      </c>
+      <c r="E26">
+        <v>508.2</v>
+      </c>
+      <c r="F26" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27">
+        <v>0.39900000000000002</v>
+      </c>
+      <c r="D27">
+        <v>0.60099999999999998</v>
+      </c>
+      <c r="E27">
+        <v>488.5</v>
+      </c>
+      <c r="F27" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28">
+        <v>0.30099999999999999</v>
+      </c>
+      <c r="D28">
+        <v>0.69900000000000007</v>
+      </c>
+      <c r="E28">
+        <v>496.9</v>
+      </c>
+      <c r="F28" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="D29">
+        <v>0.79899999999999993</v>
+      </c>
+      <c r="E29">
+        <v>515.9</v>
+      </c>
+      <c r="F29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30">
+        <v>0.10299999999999999</v>
+      </c>
+      <c r="D30">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="E30">
+        <v>527.6</v>
+      </c>
+      <c r="F30" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="D31">
+        <v>5.4000000000000048E-2</v>
+      </c>
+      <c r="E31">
+        <v>601.9</v>
+      </c>
+      <c r="F31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32">
+        <v>0.9</v>
+      </c>
+      <c r="D32">
+        <v>9.9999999999999978E-2</v>
+      </c>
+      <c r="E32">
+        <v>596.4</v>
+      </c>
+      <c r="F32" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33">
+        <v>0.80100000000000005</v>
+      </c>
+      <c r="D33">
+        <v>0.19899999999999995</v>
+      </c>
+      <c r="E33">
+        <v>563.1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34">
+        <v>0.69599999999999995</v>
+      </c>
+      <c r="D34">
+        <v>0.30400000000000005</v>
+      </c>
+      <c r="E34">
+        <v>532.29999999999995</v>
+      </c>
+      <c r="F34" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35">
+        <v>0.59899999999999998</v>
+      </c>
+      <c r="D35">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="E35">
+        <v>507.7</v>
+      </c>
+      <c r="F35" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36">
+        <v>0.5</v>
+      </c>
+      <c r="D36">
+        <v>0.5</v>
+      </c>
+      <c r="E36">
+        <v>475.7</v>
+      </c>
+      <c r="F36" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37">
+        <v>0.4</v>
+      </c>
+      <c r="D37">
+        <v>0.6</v>
+      </c>
+      <c r="E37">
+        <v>447.7</v>
+      </c>
+      <c r="F37" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38">
+        <v>0.3</v>
+      </c>
+      <c r="D38">
+        <v>0.7</v>
+      </c>
+      <c r="E38">
+        <v>459</v>
+      </c>
+      <c r="F38" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39">
+        <v>0.2</v>
+      </c>
+      <c r="D39">
+        <v>0.8</v>
+      </c>
+      <c r="E39">
+        <v>490.9</v>
+      </c>
+      <c r="F39" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40">
+        <v>0.111</v>
+      </c>
+      <c r="D40">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="E40">
+        <v>512.9</v>
+      </c>
+      <c r="F40" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="D41">
+        <v>0.93199999999999994</v>
+      </c>
+      <c r="E41">
+        <v>520.9</v>
+      </c>
+      <c r="F41" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="D42">
+        <v>5.1000000000000045E-2</v>
+      </c>
+      <c r="E42">
+        <v>603</v>
+      </c>
+      <c r="F42" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" t="s">
+        <v>92</v>
+      </c>
+      <c r="C43">
+        <v>0.89900000000000002</v>
+      </c>
+      <c r="D43">
+        <v>0.10099999999999998</v>
+      </c>
+      <c r="E43">
+        <v>589.20000000000005</v>
+      </c>
+      <c r="F43" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" t="s">
+        <v>92</v>
+      </c>
+      <c r="C44">
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="D44">
+        <v>0.20199999999999996</v>
+      </c>
+      <c r="E44">
+        <v>551.79999999999995</v>
+      </c>
+      <c r="F44" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="D45">
+        <v>0.30100000000000005</v>
+      </c>
+      <c r="E45">
+        <v>515.20000000000005</v>
+      </c>
+      <c r="F45" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" t="s">
+        <v>92</v>
+      </c>
+      <c r="C46">
+        <v>0.6</v>
+      </c>
+      <c r="D46">
+        <v>0.4</v>
+      </c>
+      <c r="E46">
+        <v>465.5</v>
+      </c>
+      <c r="F46" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" t="s">
+        <v>92</v>
+      </c>
+      <c r="C47">
+        <v>0.502</v>
+      </c>
+      <c r="D47">
+        <v>0.498</v>
+      </c>
+      <c r="E47">
+        <v>421.5</v>
+      </c>
+      <c r="F47" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" t="s">
+        <v>92</v>
+      </c>
+      <c r="C48">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="D48">
+        <v>0.59899999999999998</v>
+      </c>
+      <c r="E48">
+        <v>360.7</v>
+      </c>
+      <c r="F48" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" t="s">
+        <v>92</v>
+      </c>
+      <c r="C49">
+        <v>0.30299999999999999</v>
+      </c>
+      <c r="D49">
+        <v>0.69700000000000006</v>
+      </c>
+      <c r="E49">
+        <v>405.6</v>
+      </c>
+      <c r="F49" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="D50">
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="E50">
+        <v>439.8</v>
+      </c>
+      <c r="F50" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" t="s">
+        <v>92</v>
+      </c>
+      <c r="C51">
+        <v>0.10299999999999999</v>
+      </c>
+      <c r="D51">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="E51">
+        <v>477.5</v>
+      </c>
+      <c r="F51" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" t="s">
+        <v>92</v>
+      </c>
+      <c r="C52">
+        <v>5.5E-2</v>
+      </c>
+      <c r="D52">
+        <v>0.94499999999999995</v>
+      </c>
+      <c r="E52">
+        <v>489.7</v>
+      </c>
+      <c r="F52" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" t="s">
+        <v>94</v>
+      </c>
+      <c r="C53">
+        <v>0.65700000000000003</v>
+      </c>
+      <c r="D53">
+        <v>0.34299999999999997</v>
+      </c>
+      <c r="E53">
+        <v>873.15</v>
+      </c>
+      <c r="F53" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="D54">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="E54">
+        <v>825.15</v>
+      </c>
+      <c r="F54" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>93</v>
+      </c>
+      <c r="B55" t="s">
+        <v>94</v>
+      </c>
+      <c r="C55">
+        <v>0.57399999999999995</v>
+      </c>
+      <c r="D55">
+        <v>0.42600000000000005</v>
+      </c>
+      <c r="E55">
+        <v>800.15</v>
+      </c>
+      <c r="F55" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>93</v>
+      </c>
+      <c r="B56" t="s">
+        <v>94</v>
+      </c>
+      <c r="C56">
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="D56">
+        <v>0.47799999999999998</v>
+      </c>
+      <c r="E56">
+        <v>750.15</v>
+      </c>
+      <c r="F56" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>93</v>
+      </c>
+      <c r="B57" t="s">
+        <v>94</v>
+      </c>
+      <c r="C57">
+        <v>0.442</v>
+      </c>
+      <c r="D57">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="E57">
+        <v>658.15</v>
+      </c>
+      <c r="F57" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>93</v>
+      </c>
+      <c r="B58" t="s">
+        <v>94</v>
+      </c>
+      <c r="C58">
+        <v>0.42699999999999999</v>
+      </c>
+      <c r="D58">
+        <v>0.57299999999999995</v>
+      </c>
+      <c r="E58">
+        <v>640.15</v>
+      </c>
+      <c r="F58" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>93</v>
+      </c>
+      <c r="B59" t="s">
+        <v>94</v>
+      </c>
+      <c r="C59">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="D59">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="E59">
+        <v>636.15</v>
+      </c>
+      <c r="F59" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>93</v>
+      </c>
+      <c r="B60" t="s">
+        <v>94</v>
+      </c>
+      <c r="C60">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="D60">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="E60">
+        <v>634.15</v>
+      </c>
+      <c r="F60" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>93</v>
+      </c>
+      <c r="B61" t="s">
+        <v>94</v>
+      </c>
+      <c r="C61">
+        <v>0.41299999999999998</v>
+      </c>
+      <c r="D61">
+        <v>0.58699999999999997</v>
+      </c>
+      <c r="E61">
+        <v>635.15</v>
+      </c>
+      <c r="F61" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>93</v>
+      </c>
+      <c r="B62" t="s">
+        <v>94</v>
+      </c>
+      <c r="C62">
+        <v>0.40600000000000003</v>
+      </c>
+      <c r="D62">
+        <v>0.59399999999999997</v>
+      </c>
+      <c r="E62">
+        <v>645.15</v>
+      </c>
+      <c r="F62" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>93</v>
+      </c>
+      <c r="B63" t="s">
+        <v>94</v>
+      </c>
+      <c r="C63">
+        <v>0.38700000000000001</v>
+      </c>
+      <c r="D63">
+        <v>0.61299999999999999</v>
+      </c>
+      <c r="E63">
+        <v>661.15</v>
+      </c>
+      <c r="F63" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>93</v>
+      </c>
+      <c r="B64" t="s">
+        <v>94</v>
+      </c>
+      <c r="C64">
+        <v>0.35599999999999998</v>
+      </c>
+      <c r="D64">
+        <v>0.64400000000000002</v>
+      </c>
+      <c r="E64">
+        <v>685.15</v>
+      </c>
+      <c r="F64" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Current config of single kernal based MTGPR with optimization or single check workflows
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82934A1-3E9D-4F5D-96C2-17F125CE508B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE86318-6F99-4A86-B195-AF703703A857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-26940" yWindow="525" windowWidth="21600" windowHeight="14715" activeTab="1" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="Unfinished CATALOG" sheetId="1" r:id="rId1"/>
@@ -885,7 +885,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="220">
   <si>
     <t>Full Name</t>
   </si>
@@ -1215,6 +1215,339 @@
   </si>
   <si>
     <t>K</t>
+  </si>
+  <si>
+    <t>lithium borohydride</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium borohydride</t>
+  </si>
+  <si>
+    <t>ammonia borane</t>
+  </si>
+  <si>
+    <t>thiourea</t>
+  </si>
+  <si>
+    <t>thioacetamide</t>
+  </si>
+  <si>
+    <t>acetonitrile</t>
+  </si>
+  <si>
+    <t>CC#N</t>
+  </si>
+  <si>
+    <t>ammonia</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>benzonitrile</t>
+  </si>
+  <si>
+    <t>C1=CC=C(C=C1)C#N</t>
+  </si>
+  <si>
+    <t>boron</t>
+  </si>
+  <si>
+    <t>[B]</t>
+  </si>
+  <si>
+    <t>butanenitrile</t>
+  </si>
+  <si>
+    <t>CCCC#N</t>
+  </si>
+  <si>
+    <t>calcium</t>
+  </si>
+  <si>
+    <t>[Ca]</t>
+  </si>
+  <si>
+    <t>calcium nitrate</t>
+  </si>
+  <si>
+    <t>[N+](=O)([O-])[O-].[N+](=O)([O-])[O-].[Ca+2]</t>
+  </si>
+  <si>
+    <t>carbon</t>
+  </si>
+  <si>
+    <t>[C]</t>
+  </si>
+  <si>
+    <t>cesium chloride</t>
+  </si>
+  <si>
+    <t>[Cl-].[Cs+]</t>
+  </si>
+  <si>
+    <t>cyanogen</t>
+  </si>
+  <si>
+    <t>C(#N)C#N</t>
+  </si>
+  <si>
+    <t>dichlorine</t>
+  </si>
+  <si>
+    <t>ClCl</t>
+  </si>
+  <si>
+    <t>dihydrogen</t>
+  </si>
+  <si>
+    <t>[H][H]</t>
+  </si>
+  <si>
+    <t>dimethylamine</t>
+  </si>
+  <si>
+    <t>CNC</t>
+  </si>
+  <si>
+    <t>dimethylhydrazine</t>
+  </si>
+  <si>
+    <t>CN(C)N</t>
+  </si>
+  <si>
+    <t>dinitrogen</t>
+  </si>
+  <si>
+    <t>N#N</t>
+  </si>
+  <si>
+    <t>dinitrogen tetroxide</t>
+  </si>
+  <si>
+    <t>[N+](=O)([N+](=O)[O-])[O-]</t>
+  </si>
+  <si>
+    <t>dioxygen</t>
+  </si>
+  <si>
+    <t>O=O</t>
+  </si>
+  <si>
+    <t>ethane</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>ethyl bromide</t>
+  </si>
+  <si>
+    <t>CCBr</t>
+  </si>
+  <si>
+    <t>ethyl chloride</t>
+  </si>
+  <si>
+    <t>CCCl</t>
+  </si>
+  <si>
+    <t>ethyl iodide</t>
+  </si>
+  <si>
+    <t>CCI</t>
+  </si>
+  <si>
+    <t>hydrazine</t>
+  </si>
+  <si>
+    <t>NN</t>
+  </si>
+  <si>
+    <t>lithium</t>
+  </si>
+  <si>
+    <t>[Li]</t>
+  </si>
+  <si>
+    <t>methane</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>methyl bromide</t>
+  </si>
+  <si>
+    <t>CBr</t>
+  </si>
+  <si>
+    <t>methyl chloride</t>
+  </si>
+  <si>
+    <t>CCl</t>
+  </si>
+  <si>
+    <t>methyl iodide</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>methylamine</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>monomethylhydrazine</t>
+  </si>
+  <si>
+    <t>CNN</t>
+  </si>
+  <si>
+    <t>potassium</t>
+  </si>
+  <si>
+    <t>[K]</t>
+  </si>
+  <si>
+    <t>potassium nitrate</t>
+  </si>
+  <si>
+    <t>[N+](=O)([O-])[O-].[K+]</t>
+  </si>
+  <si>
+    <t>propanenitrile</t>
+  </si>
+  <si>
+    <t>CCC#N</t>
+  </si>
+  <si>
+    <t>propylamine</t>
+  </si>
+  <si>
+    <t>CCCN</t>
+  </si>
+  <si>
+    <t>rubidium chloride</t>
+  </si>
+  <si>
+    <t>[Cl-].[Rb+]</t>
+  </si>
+  <si>
+    <t>sodium</t>
+  </si>
+  <si>
+    <t>[Na]</t>
+  </si>
+  <si>
+    <t>sodium chloride</t>
+  </si>
+  <si>
+    <t>[Na+].[Cl-]</t>
+  </si>
+  <si>
+    <t>sodium nitrate</t>
+  </si>
+  <si>
+    <t>[N+](=O)([O-])[O-].[Na+]</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium bromide</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[Br-]</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium iodide</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[I-]</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium nitrate</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[N+](=O)([O-])[O-]</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium tetraphenylborate</t>
+  </si>
+  <si>
+    <t>[B-](C1=CC=CC=C1)(C2=CC=CC=C2)(C3=CC=CC=C3)C4=CC=CC=C4.CCCC[N+](CCCC)(CCCC)CCCC</t>
+  </si>
+  <si>
+    <t>tetraethylammonium iodide</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[I-]</t>
+  </si>
+  <si>
+    <t>tetraethylammonium nitrate</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[N+](=O)([O-])[O-]</t>
+  </si>
+  <si>
+    <t>tetraheptylammonium chloride</t>
+  </si>
+  <si>
+    <t>CCCCCCC[N+](CCCCCCC)(CCCCCCC)CCCCCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>tetrahexylammonium bromide</t>
+  </si>
+  <si>
+    <t>CCCCCC[N+](CCCCCC)(CCCCCC)CCCCCC.[Br-]</t>
+  </si>
+  <si>
+    <t>tetramethylammonium bromide</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[Br-]</t>
+  </si>
+  <si>
+    <t>tetramethylammonium iodide</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[I-]</t>
+  </si>
+  <si>
+    <t>tetramethylammonium nitrate</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[N+](=O)([O-])[O-]</t>
+  </si>
+  <si>
+    <t>tetrapentylammonium bromide</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[Br-]</t>
+  </si>
+  <si>
+    <t>tetrapentylammonium chloride</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>tetrapentylammonium iodide</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[I-]</t>
+  </si>
+  <si>
+    <t>tetrapropylammonium iodide</t>
+  </si>
+  <si>
+    <t>CCC[N+](CCC)(CCC)CCC.[I-]</t>
+  </si>
+  <si>
+    <t>trimethylamine</t>
+  </si>
+  <si>
+    <t>CN(C)C</t>
   </si>
 </sst>
 </file>
@@ -1269,7 +1602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1282,6 +1615,11 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2180,7 +2518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE786A1-84C7-4241-A3B9-138356725320}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.28515625" bestFit="1" customWidth="1"/>
@@ -2235,67 +2573,597 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="A2" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B59" s="6"/>
+      <c r="C59" s="6" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B60" s="6"/>
+      <c r="C60" s="6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>94</v>
-      </c>
-      <c r="C9" t="s">
-        <v>101</v>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B63" s="8"/>
+      <c r="C63" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="8"/>
+      <c r="C64" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B65" s="8"/>
+      <c r="C65" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>